<commit_message>
Resolve Naive display landing and fabrication rules; add bring-up tools
</commit_message>
<xml_diff>
--- a/1.Hardware/RevB-KiCad/Naive/BOM.xlsx
+++ b/1.Hardware/RevB-KiCad/Naive/BOM.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采购清单" sheetId="1" r:id="Rab033e6e49e8463d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装配明细" sheetId="2" r:id="Ra6fc967c388f4e30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采购清单" sheetId="1" r:id="R4ef75d9112684647"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装配明细" sheetId="2" r:id="Rc90cf3caab1f4799"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -606,7 +606,7 @@
         <x:v>电气候选，机械待验收</x:v>
       </x:c>
       <x:c r="G10" s="4" t="str">
-        <x:v>裸屏12pin/0.7mm/ST7789V；尾排绕板、焊盘注册及整壳装配须样件确认</x:v>
+        <x:v>12pin/0.7mm/ST7789V；5.5x0.5mm无F.Paste长焊盘，PCBA后手工焊FPC；仅核纵向落点，折弯/接触面/整壳仍待样件</x:v>
       </x:c>
       <x:c r="H10" s="2"/>
       <x:c r="I10" s="2"/>
@@ -1913,7 +1913,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44a27316b47445e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R745ed9cb43db48b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4022,7 +4022,7 @@
         <x:v>电气候选，机械待验收</x:v>
       </x:c>
       <x:c r="I70" s="4" t="str">
-        <x:v>裸屏12pin/0.7mm/ST7789V；尾排绕板、焊盘注册及整壳装配须样件确认</x:v>
+        <x:v>12pin/0.7mm/ST7789V；5.5x0.5mm无F.Paste长焊盘，PCBA后手工焊FPC；仅核纵向落点，折弯/接触面/整壳仍待样件</x:v>
       </x:c>
       <x:c r="J70" s="4" t="str">
         <x:v>https://www.polcd-digital.com/products/1-3-inch-tft-lcd-display-240x240-pixels-p133h002</x:v>
@@ -4190,7 +4190,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdc26400945a4de6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b16560253fa498c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Use compatible small-quantity parts in Naive RevB
</commit_message>
<xml_diff>
--- a/1.Hardware/RevB-KiCad/Naive/BOM.xlsx
+++ b/1.Hardware/RevB-KiCad/Naive/BOM.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采购清单" sheetId="1" r:id="R4ef75d9112684647"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装配明细" sheetId="2" r:id="Rc90cf3caab1f4799"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采购清单" sheetId="1" r:id="Re5426e4c7ff34047"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装配明细" sheetId="2" r:id="Rae51f4aa81f94e5a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -172,8 +172,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PurchasingParts" displayName="PurchasingParts" ref="A6:G45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:G45"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PurchasingParts" displayName="PurchasingParts" ref="A6:G44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:G44"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="完整订货号 MPN"/>
     <x:tableColumn id="2" name="厂家"/>
@@ -429,7 +429,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>2026-10-29  每台两块PCB的装配用量</x:v>
+        <x:v>2026-10-30  每台两块PCB的装配用量</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -456,7 +456,7 @@
         <x:v>订货型号数</x:v>
       </x:c>
       <x:c r="E4" s="2" t="n">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="F4" s="2"/>
       <x:c r="G4" s="2" t="str">
@@ -969,26 +969,28 @@
     </x:row>
     <x:row r="24" ht="54" customHeight="1">
       <x:c r="A24" s="5" t="str">
-        <x:v>GRM188R71A105KA61D</x:v>
+        <x:v>GRM188R71E105KA12D</x:v>
       </x:c>
       <x:c r="B24" s="5" t="str">
         <x:v>Murata</x:v>
       </x:c>
       <x:c r="C24" s="6" t="n">
         <x:f>SUMIFS('装配明细'!$C$7:$C$75,'装配明细'!$E$7:$E$75,A24)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D24" s="4" t="str">
         <x:v>1uF</x:v>
       </x:c>
       <x:c r="E24" s="4" t="str">
-        <x:v>屏板: C4</x:v>
+        <x:v>主板: C24
+屏板: C4</x:v>
       </x:c>
       <x:c r="F24" s="4" t="str">
         <x:v>原理图已选完整MPN</x:v>
       </x:c>
       <x:c r="G24" s="4" t="str">
-        <x:v>MLCC标称值不代表工作偏压下有效值</x:v>
+        <x:v>25V/1uF/X7R±10%/0603；与ExtendBoard:C4同料C86020，各焊1颗；BH1750 DVI保留R11=1k，冷启动/快速重启时序须实测
+25V/1uF/X7R±10%/0603；5V本地旁路，与MainBoard:C24同料C86020，各焊1颗；供电与热插拔须实测</x:v>
       </x:c>
       <x:c r="H24" s="2"/>
       <x:c r="I24" s="2"/>
@@ -996,7 +998,7 @@
     </x:row>
     <x:row r="25" ht="54" customHeight="1">
       <x:c r="A25" s="5" t="str">
-        <x:v>GRM188R71C105KA12D</x:v>
+        <x:v>GRM1555C1H101JA01D</x:v>
       </x:c>
       <x:c r="B25" s="5" t="str">
         <x:v>Murata</x:v>
@@ -1006,16 +1008,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D25" s="4" t="str">
-        <x:v>1uF</x:v>
+        <x:v>100pF</x:v>
       </x:c>
       <x:c r="E25" s="4" t="str">
-        <x:v>主板: C24</x:v>
+        <x:v>主板: C16</x:v>
       </x:c>
       <x:c r="F25" s="4" t="str">
         <x:v>原理图已选完整MPN</x:v>
       </x:c>
       <x:c r="G25" s="4" t="str">
-        <x:v>MLCC标称值不代表工作偏压下有效值</x:v>
+        <x:v>100pF/50V/C0G±5%0402；TI Eq3估算约0.425ms@5V，非最大值保证；CP_VDD到2.7V≤1ms、热插拔与入口电流须实测</x:v>
       </x:c>
       <x:c r="H25" s="2"/>
       <x:c r="I25" s="2"/>
@@ -1023,7 +1025,7 @@
     </x:row>
     <x:row r="26" ht="54" customHeight="1">
       <x:c r="A26" s="5" t="str">
-        <x:v>GRM1555C1H101JA01D</x:v>
+        <x:v>GRM1555C1H222JA01D</x:v>
       </x:c>
       <x:c r="B26" s="5" t="str">
         <x:v>Murata</x:v>
@@ -1033,16 +1035,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D26" s="4" t="str">
-        <x:v>100pF</x:v>
+        <x:v>2.2nF</x:v>
       </x:c>
       <x:c r="E26" s="4" t="str">
-        <x:v>主板: C16</x:v>
+        <x:v>主板: C9</x:v>
       </x:c>
       <x:c r="F26" s="4" t="str">
         <x:v>原理图已选完整MPN</x:v>
       </x:c>
       <x:c r="G26" s="4" t="str">
-        <x:v>100pF/50V/C0G±5%0402；TI Eq3估算约0.425ms@5V，非最大值保证；CP_VDD到2.7V≤1ms、热插拔与入口电流须实测</x:v>
+        <x:v>MLCC标称值不代表工作偏压下有效值</x:v>
       </x:c>
       <x:c r="H26" s="2"/>
       <x:c r="I26" s="2"/>
@@ -1050,26 +1052,26 @@
     </x:row>
     <x:row r="27" ht="54" customHeight="1">
       <x:c r="A27" s="5" t="str">
-        <x:v>GRM1555C1H222JA01D</x:v>
+        <x:v>MMBT3904-7-F</x:v>
       </x:c>
       <x:c r="B27" s="5" t="str">
-        <x:v>Murata</x:v>
+        <x:v>Diodes Incorporated</x:v>
       </x:c>
       <x:c r="C27" s="6" t="n">
         <x:f>SUMIFS('装配明细'!$C$7:$C$75,'装配明细'!$E$7:$E$75,A27)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D27" s="4" t="str">
-        <x:v>2.2nF</x:v>
+        <x:v>MMBT3904-7-F</x:v>
       </x:c>
       <x:c r="E27" s="4" t="str">
-        <x:v>主板: C9</x:v>
+        <x:v>主板: VT1, VT2</x:v>
       </x:c>
       <x:c r="F27" s="4" t="str">
-        <x:v>原理图已选完整MPN</x:v>
+        <x:v>厂家图纸已核</x:v>
       </x:c>
       <x:c r="G27" s="4" t="str">
-        <x:v>MLCC标称值不代表工作偏压下有效值</x:v>
+        <x:v>B1/E2/C3；按Diodes受控SOT23焊盘，不任意替换不同引脚8050</x:v>
       </x:c>
       <x:c r="H27" s="2"/>
       <x:c r="I27" s="2"/>
@@ -1077,34 +1079,33 @@
     </x:row>
     <x:row r="28" ht="54" customHeight="1">
       <x:c r="A28" s="5" t="str">
-        <x:v>MMBT3904-7-F</x:v>
+        <x:v>RC0402FR-071KL</x:v>
       </x:c>
       <x:c r="B28" s="5" t="str">
-        <x:v>Diodes Incorporated</x:v>
+        <x:v>YAGEO</x:v>
       </x:c>
       <x:c r="C28" s="6" t="n">
         <x:f>SUMIFS('装配明细'!$C$7:$C$75,'装配明细'!$E$7:$E$75,A28)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D28" s="4" t="str">
-        <x:v>MMBT3904-7-F</x:v>
+        <x:v>1k</x:v>
       </x:c>
       <x:c r="E28" s="4" t="str">
-        <x:v>主板: VT1, VT2</x:v>
+        <x:v>主板: R11
+屏板: R1</x:v>
       </x:c>
       <x:c r="F28" s="4" t="str">
-        <x:v>厂家图纸已核</x:v>
-      </x:c>
-      <x:c r="G28" s="4" t="str">
-        <x:v>B1/E2/C3；按Diodes受控SOT23焊盘，不任意替换不同引脚8050</x:v>
-      </x:c>
+        <x:v>未单独核验生命周期</x:v>
+      </x:c>
+      <x:c r="G28" s="4" t="str"/>
       <x:c r="H28" s="2"/>
       <x:c r="I28" s="2"/>
       <x:c r="J28" s="2"/>
     </x:row>
     <x:row r="29" ht="54" customHeight="1">
       <x:c r="A29" s="5" t="str">
-        <x:v>RC0402FR-071KL</x:v>
+        <x:v>RC0402FR-074K7L</x:v>
       </x:c>
       <x:c r="B29" s="5" t="str">
         <x:v>YAGEO</x:v>
@@ -1114,11 +1115,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="D29" s="4" t="str">
-        <x:v>1k</x:v>
+        <x:v>4.7k</x:v>
       </x:c>
       <x:c r="E29" s="4" t="str">
-        <x:v>主板: R11
-屏板: R1</x:v>
+        <x:v>主板: R14, R15</x:v>
       </x:c>
       <x:c r="F29" s="4" t="str">
         <x:v>未单独核验生命周期</x:v>
@@ -1130,7 +1130,7 @@
     </x:row>
     <x:row r="30" ht="54" customHeight="1">
       <x:c r="A30" s="5" t="str">
-        <x:v>RC0402FR-074K7L</x:v>
+        <x:v>RC0402FR-075K1L</x:v>
       </x:c>
       <x:c r="B30" s="5" t="str">
         <x:v>YAGEO</x:v>
@@ -1140,10 +1140,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="D30" s="4" t="str">
-        <x:v>4.7k</x:v>
+        <x:v>5.1k</x:v>
       </x:c>
       <x:c r="E30" s="4" t="str">
-        <x:v>主板: R14, R15</x:v>
+        <x:v>主板: R12, R13</x:v>
       </x:c>
       <x:c r="F30" s="4" t="str">
         <x:v>未单独核验生命周期</x:v>
@@ -1155,20 +1155,20 @@
     </x:row>
     <x:row r="31" ht="54" customHeight="1">
       <x:c r="A31" s="5" t="str">
-        <x:v>RC0402FR-075K1L</x:v>
+        <x:v>RC0402FR-0710KL</x:v>
       </x:c>
       <x:c r="B31" s="5" t="str">
         <x:v>YAGEO</x:v>
       </x:c>
       <x:c r="C31" s="6" t="n">
         <x:f>SUMIFS('装配明细'!$C$7:$C$75,'装配明细'!$E$7:$E$75,A31)</x:f>
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D31" s="4" t="str">
-        <x:v>5.1k</x:v>
+        <x:v>10K / 10k</x:v>
       </x:c>
       <x:c r="E31" s="4" t="str">
-        <x:v>主板: R12, R13</x:v>
+        <x:v>主板: R1, R6, R7, R8, R9, R10, R16, R17</x:v>
       </x:c>
       <x:c r="F31" s="4" t="str">
         <x:v>未单独核验生命周期</x:v>
@@ -1180,20 +1180,20 @@
     </x:row>
     <x:row r="32" ht="54" customHeight="1">
       <x:c r="A32" s="5" t="str">
-        <x:v>RC0402FR-0710KL</x:v>
+        <x:v>RC0402FR-0712KL</x:v>
       </x:c>
       <x:c r="B32" s="5" t="str">
         <x:v>YAGEO</x:v>
       </x:c>
       <x:c r="C32" s="6" t="n">
         <x:f>SUMIFS('装配明细'!$C$7:$C$75,'装配明细'!$E$7:$E$75,A32)</x:f>
-        <x:v>8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D32" s="4" t="str">
-        <x:v>10K / 10k</x:v>
+        <x:v>12K</x:v>
       </x:c>
       <x:c r="E32" s="4" t="str">
-        <x:v>主板: R1, R6, R7, R8, R9, R10, R16, R17</x:v>
+        <x:v>主板: R4, R5</x:v>
       </x:c>
       <x:c r="F32" s="4" t="str">
         <x:v>未单独核验生命周期</x:v>
@@ -1205,20 +1205,20 @@
     </x:row>
     <x:row r="33" ht="54" customHeight="1">
       <x:c r="A33" s="5" t="str">
-        <x:v>RC0402FR-0712KL</x:v>
+        <x:v>RC0402FR-0733RL</x:v>
       </x:c>
       <x:c r="B33" s="5" t="str">
         <x:v>YAGEO</x:v>
       </x:c>
       <x:c r="C33" s="6" t="n">
         <x:f>SUMIFS('装配明细'!$C$7:$C$75,'装配明细'!$E$7:$E$75,A33)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D33" s="4" t="str">
-        <x:v>12K</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E33" s="4" t="str">
-        <x:v>主板: R4, R5</x:v>
+        <x:v>主板: R20</x:v>
       </x:c>
       <x:c r="F33" s="4" t="str">
         <x:v>未单独核验生命周期</x:v>
@@ -1230,20 +1230,21 @@
     </x:row>
     <x:row r="34" ht="54" customHeight="1">
       <x:c r="A34" s="5" t="str">
-        <x:v>RC0402FR-0733RL</x:v>
+        <x:v>RC0402FR-07100KL</x:v>
       </x:c>
       <x:c r="B34" s="5" t="str">
         <x:v>YAGEO</x:v>
       </x:c>
       <x:c r="C34" s="6" t="n">
         <x:f>SUMIFS('装配明细'!$C$7:$C$75,'装配明细'!$E$7:$E$75,A34)</x:f>
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D34" s="4" t="str">
-        <x:v>33</x:v>
+        <x:v>100k</x:v>
       </x:c>
       <x:c r="E34" s="4" t="str">
-        <x:v>主板: R20</x:v>
+        <x:v>主板: R18, R19
+屏板: R3</x:v>
       </x:c>
       <x:c r="F34" s="4" t="str">
         <x:v>未单独核验生命周期</x:v>
@@ -1255,33 +1256,34 @@
     </x:row>
     <x:row r="35" ht="54" customHeight="1">
       <x:c r="A35" s="5" t="str">
-        <x:v>RC0402FR-07100KL</x:v>
+        <x:v>RC0402JR-070RL</x:v>
       </x:c>
       <x:c r="B35" s="5" t="str">
         <x:v>YAGEO</x:v>
       </x:c>
       <x:c r="C35" s="6" t="n">
         <x:f>SUMIFS('装配明细'!$C$7:$C$75,'装配明细'!$E$7:$E$75,A35)</x:f>
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D35" s="4" t="str">
-        <x:v>100k</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E35" s="4" t="str">
-        <x:v>主板: R18, R19
-屏板: R3</x:v>
+        <x:v>主板: R2</x:v>
       </x:c>
       <x:c r="F35" s="4" t="str">
         <x:v>未单独核验生命周期</x:v>
       </x:c>
-      <x:c r="G35" s="4" t="str"/>
+      <x:c r="G35" s="4" t="str">
+        <x:v>0ohm0402，型号额定1A；3V3A支路按ESP≤500mA设计分配</x:v>
+      </x:c>
       <x:c r="H35" s="2"/>
       <x:c r="I35" s="2"/>
       <x:c r="J35" s="2"/>
     </x:row>
     <x:row r="36" ht="54" customHeight="1">
       <x:c r="A36" s="5" t="str">
-        <x:v>RC0402FR-07200RL</x:v>
+        <x:v>RC0603FR-0727RL</x:v>
       </x:c>
       <x:c r="B36" s="5" t="str">
         <x:v>YAGEO</x:v>
@@ -1291,10 +1293,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D36" s="4" t="str">
-        <x:v>200R</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E36" s="4" t="str">
-        <x:v>主板: R3</x:v>
+        <x:v>屏板: R2</x:v>
       </x:c>
       <x:c r="F36" s="4" t="str">
         <x:v>未单独核验生命周期</x:v>
@@ -1306,26 +1308,26 @@
     </x:row>
     <x:row r="37" ht="54" customHeight="1">
       <x:c r="A37" s="5" t="str">
-        <x:v>RC0402JR-070RL</x:v>
+        <x:v>RTT022000FTH</x:v>
       </x:c>
       <x:c r="B37" s="5" t="str">
-        <x:v>YAGEO</x:v>
+        <x:v>RALEC</x:v>
       </x:c>
       <x:c r="C37" s="6" t="n">
         <x:f>SUMIFS('装配明细'!$C$7:$C$75,'装配明细'!$E$7:$E$75,A37)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D37" s="4" t="str">
-        <x:v>0</x:v>
+        <x:v>200R</x:v>
       </x:c>
       <x:c r="E37" s="4" t="str">
-        <x:v>主板: R2</x:v>
+        <x:v>主板: R3</x:v>
       </x:c>
       <x:c r="F37" s="4" t="str">
-        <x:v>未单独核验生命周期</x:v>
+        <x:v>原厂规格已核</x:v>
       </x:c>
       <x:c r="G37" s="4" t="str">
-        <x:v>0ohm0402，型号额定1A；3V3A支路按ESP≤500mA设计分配</x:v>
+        <x:v>UART串联200ohm±1%/0402；原位兼容；现有密集land与原厂推荐图有差异，落锡/贴装工艺须验收</x:v>
       </x:c>
       <x:c r="H37" s="2"/>
       <x:c r="I37" s="2"/>
@@ -1333,32 +1335,34 @@
     </x:row>
     <x:row r="38" ht="54" customHeight="1">
       <x:c r="A38" s="5" t="str">
-        <x:v>RC0603FR-0727RL</x:v>
+        <x:v>SN74AHCT1G125DCKR</x:v>
       </x:c>
       <x:c r="B38" s="5" t="str">
-        <x:v>YAGEO</x:v>
+        <x:v>Texas Instruments</x:v>
       </x:c>
       <x:c r="C38" s="6" t="n">
         <x:f>SUMIFS('装配明细'!$C$7:$C$75,'装配明细'!$E$7:$E$75,A38)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D38" s="4" t="str">
-        <x:v>27</x:v>
+        <x:v>SN74AHCT1G125DCKR</x:v>
       </x:c>
       <x:c r="E38" s="4" t="str">
-        <x:v>屏板: R2</x:v>
+        <x:v>主板: U8</x:v>
       </x:c>
       <x:c r="F38" s="4" t="str">
-        <x:v>未单独核验生命周期</x:v>
-      </x:c>
-      <x:c r="G38" s="4" t="str"/>
+        <x:v>Active（原厂）</x:v>
+      </x:c>
+      <x:c r="G38" s="4" t="str">
+        <x:v>保持完整封装后缀与引脚定义</x:v>
+      </x:c>
       <x:c r="H38" s="2"/>
       <x:c r="I38" s="2"/>
       <x:c r="J38" s="2"/>
     </x:row>
     <x:row r="39" ht="54" customHeight="1">
       <x:c r="A39" s="5" t="str">
-        <x:v>SN74AHCT1G125DCKR</x:v>
+        <x:v>TPD1E10B06DPYR</x:v>
       </x:c>
       <x:c r="B39" s="5" t="str">
         <x:v>Texas Instruments</x:v>
@@ -1368,10 +1372,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D39" s="4" t="str">
-        <x:v>SN74AHCT1G125DCKR</x:v>
+        <x:v>TPD1E10B06DPYR</x:v>
       </x:c>
       <x:c r="E39" s="4" t="str">
-        <x:v>主板: U8</x:v>
+        <x:v>主板: D2</x:v>
       </x:c>
       <x:c r="F39" s="4" t="str">
         <x:v>Active（原厂）</x:v>
@@ -1385,7 +1389,7 @@
     </x:row>
     <x:row r="40" ht="54" customHeight="1">
       <x:c r="A40" s="5" t="str">
-        <x:v>TPD1E10B06DPYR</x:v>
+        <x:v>TPD4E05U06DQAR</x:v>
       </x:c>
       <x:c r="B40" s="5" t="str">
         <x:v>Texas Instruments</x:v>
@@ -1395,10 +1399,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D40" s="4" t="str">
-        <x:v>TPD1E10B06DPYR</x:v>
+        <x:v>TPD4E05U06DQAR</x:v>
       </x:c>
       <x:c r="E40" s="4" t="str">
-        <x:v>主板: D2</x:v>
+        <x:v>主板: U7</x:v>
       </x:c>
       <x:c r="F40" s="4" t="str">
         <x:v>Active（原厂）</x:v>
@@ -1412,7 +1416,7 @@
     </x:row>
     <x:row r="41" ht="54" customHeight="1">
       <x:c r="A41" s="5" t="str">
-        <x:v>TPD4E05U06DQAR</x:v>
+        <x:v>TPS22918DBVT</x:v>
       </x:c>
       <x:c r="B41" s="5" t="str">
         <x:v>Texas Instruments</x:v>
@@ -1422,16 +1426,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D41" s="4" t="str">
-        <x:v>TPD4E05U06DQAR</x:v>
+        <x:v>TPS22918DBVT</x:v>
       </x:c>
       <x:c r="E41" s="4" t="str">
-        <x:v>主板: U7</x:v>
+        <x:v>主板: U6</x:v>
       </x:c>
       <x:c r="F41" s="4" t="str">
         <x:v>Active（原厂）</x:v>
       </x:c>
       <x:c r="G41" s="4" t="str">
-        <x:v>保持完整封装后缀与引脚定义</x:v>
+        <x:v>同TPS22918芯片及DBV6脚；T为250pcs小盘，ON/CT网络不变；2026-10-30嘉立创需订货（渠道快照，库存/交期下单复核）</x:v>
       </x:c>
       <x:c r="H41" s="2"/>
       <x:c r="I41" s="2"/>
@@ -1439,7 +1443,7 @@
     </x:row>
     <x:row r="42" ht="54" customHeight="1">
       <x:c r="A42" s="5" t="str">
-        <x:v>TPS22918DBVR</x:v>
+        <x:v>TPS62162DSGR</x:v>
       </x:c>
       <x:c r="B42" s="5" t="str">
         <x:v>Texas Instruments</x:v>
@@ -1449,10 +1453,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D42" s="4" t="str">
-        <x:v>TPS22918DBVR</x:v>
+        <x:v>TPS62162DSGR</x:v>
       </x:c>
       <x:c r="E42" s="4" t="str">
-        <x:v>主板: U6</x:v>
+        <x:v>主板: U2</x:v>
       </x:c>
       <x:c r="F42" s="4" t="str">
         <x:v>Active（原厂）</x:v>
@@ -1466,26 +1470,26 @@
     </x:row>
     <x:row r="43" ht="54" customHeight="1">
       <x:c r="A43" s="5" t="str">
-        <x:v>TPS62162DSGR</x:v>
+        <x:v>VLS3012HBX-2R2M-N</x:v>
       </x:c>
       <x:c r="B43" s="5" t="str">
-        <x:v>Texas Instruments</x:v>
+        <x:v>TDK</x:v>
       </x:c>
       <x:c r="C43" s="6" t="n">
         <x:f>SUMIFS('装配明细'!$C$7:$C$75,'装配明细'!$E$7:$E$75,A43)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D43" s="4" t="str">
-        <x:v>TPS62162DSGR</x:v>
+        <x:v>2.2uH</x:v>
       </x:c>
       <x:c r="E43" s="4" t="str">
-        <x:v>主板: U2</x:v>
+        <x:v>主板: L1</x:v>
       </x:c>
       <x:c r="F43" s="4" t="str">
-        <x:v>Active（原厂）</x:v>
+        <x:v>未单独核验生命周期</x:v>
       </x:c>
       <x:c r="G43" s="4" t="str">
-        <x:v>保持完整封装后缀与引脚定义</x:v>
+        <x:v>2.2uH；完整HBX/-N订货号，电感饱和及温升按供电实测验收</x:v>
       </x:c>
       <x:c r="H43" s="2"/>
       <x:c r="I43" s="2"/>
@@ -1493,54 +1497,39 @@
     </x:row>
     <x:row r="44" ht="54" customHeight="1">
       <x:c r="A44" s="5" t="str">
-        <x:v>VLS3012HBX-2R2M-N</x:v>
+        <x:v>WS2812B-V5/W</x:v>
       </x:c>
       <x:c r="B44" s="5" t="str">
-        <x:v>TDK</x:v>
+        <x:v>Worldsemi</x:v>
       </x:c>
       <x:c r="C44" s="6" t="n">
         <x:f>SUMIFS('装配明细'!$C$7:$C$75,'装配明细'!$E$7:$E$75,A44)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D44" s="4" t="str">
-        <x:v>2.2uH</x:v>
+        <x:v>WS2812B-V5/W</x:v>
       </x:c>
       <x:c r="E44" s="4" t="str">
-        <x:v>主板: L1</x:v>
+        <x:v>主板: D1</x:v>
       </x:c>
       <x:c r="F44" s="4" t="str">
-        <x:v>未单独核验生命周期</x:v>
+        <x:v>厂家资料已核</x:v>
       </x:c>
       <x:c r="G44" s="4" t="str">
-        <x:v>2.2uH；完整HBX/-N订货号，电感饱和及温升按供电实测验收</x:v>
+        <x:v>完整V5/W版本；1VDD/2DOUT/3GND/4DIN；5V供电及AHCT缓冲</x:v>
       </x:c>
       <x:c r="H44" s="2"/>
       <x:c r="I44" s="2"/>
       <x:c r="J44" s="2"/>
     </x:row>
-    <x:row r="45" ht="54" customHeight="1">
-      <x:c r="A45" s="5" t="str">
-        <x:v>WS2812B-V5/W</x:v>
-      </x:c>
-      <x:c r="B45" s="5" t="str">
-        <x:v>Worldsemi</x:v>
-      </x:c>
-      <x:c r="C45" s="6" t="n">
-        <x:f>SUMIFS('装配明细'!$C$7:$C$75,'装配明细'!$E$7:$E$75,A45)</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D45" s="4" t="str">
-        <x:v>WS2812B-V5/W</x:v>
-      </x:c>
-      <x:c r="E45" s="4" t="str">
-        <x:v>主板: D1</x:v>
-      </x:c>
-      <x:c r="F45" s="4" t="str">
-        <x:v>厂家资料已核</x:v>
-      </x:c>
-      <x:c r="G45" s="4" t="str">
-        <x:v>完整V5/W版本；1VDD/2DOUT/3GND/4DIN；5V供电及AHCT缓冲</x:v>
-      </x:c>
+    <x:row r="45">
+      <x:c r="A45" s="2"/>
+      <x:c r="B45" s="2"/>
+      <x:c r="C45" s="2"/>
+      <x:c r="D45" s="2"/>
+      <x:c r="E45" s="2"/>
+      <x:c r="F45" s="2"/>
+      <x:c r="G45" s="2"/>
       <x:c r="H45" s="2"/>
       <x:c r="I45" s="2"/>
       <x:c r="J45" s="2"/>
@@ -1906,14 +1895,14 @@
       <x:c r="J75" s="2"/>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="F7:F45">
+  <x:conditionalFormatting sqref="F7:F44">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Obsolete"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="NRND"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="待验收"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R745ed9cb43db48b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb99d970ac1044ff8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1950,7 +1939,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>2026-10-29  每行对应一个实际位号，数量单位：件/台</x:v>
+        <x:v>2026-10-30  每行对应一个实际位号，数量单位：件/台</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2706,7 +2695,7 @@
         <x:v>1uF</x:v>
       </x:c>
       <x:c r="E28" s="7" t="str">
-        <x:v>GRM188R71C105KA12D</x:v>
+        <x:v>GRM188R71E105KA12D</x:v>
       </x:c>
       <x:c r="F28" s="7" t="str">
         <x:v>Murata</x:v>
@@ -2718,10 +2707,10 @@
         <x:v>原理图已选完整MPN</x:v>
       </x:c>
       <x:c r="I28" s="4" t="str">
-        <x:v>MLCC标称值不代表工作偏压下有效值</x:v>
+        <x:v>25V/1uF/X7R±10%/0603；与ExtendBoard:C4同料C86020，各焊1颗；BH1750 DVI保留R11=1k，冷启动/快速重启时序须实测</x:v>
       </x:c>
       <x:c r="J28" s="4" t="str">
-        <x:v>https://ds.murata.com/simserve/characteristics?ReqType=TechPDF&amp;partnumber=GRM188R71C105KA12&amp;techpdfname=technical_pdf_Capacitor01&amp;lang=en</x:v>
+        <x:v>https://ds.murata.com/simserve/characteristics?ReqType=TechPDF&amp;partnumber=GRM188R71E105KA12&amp;techpdfname=technical_pdf_Capacitor01&amp;lang=en</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -2958,20 +2947,22 @@
         <x:v>200R</x:v>
       </x:c>
       <x:c r="E36" s="7" t="str">
-        <x:v>RC0402FR-07200RL</x:v>
+        <x:v>RTT022000FTH</x:v>
       </x:c>
       <x:c r="F36" s="7" t="str">
-        <x:v>YAGEO</x:v>
+        <x:v>RALEC</x:v>
       </x:c>
       <x:c r="G36" s="7" t="str">
         <x:v>HoloCubic_RevB:Original_R3</x:v>
       </x:c>
       <x:c r="H36" s="4" t="str">
-        <x:v>未单独核验生命周期</x:v>
-      </x:c>
-      <x:c r="I36" s="4" t="str"/>
+        <x:v>原厂规格已核</x:v>
+      </x:c>
+      <x:c r="I36" s="4" t="str">
+        <x:v>UART串联200ohm±1%/0402；原位兼容；现有密集land与原厂推荐图有差异，落锡/贴装工艺须验收</x:v>
+      </x:c>
       <x:c r="J36" s="4" t="str">
-        <x:v>https://www.yageogroup.com/component-documentation/download/specsheet/RC0402FR-07200RL</x:v>
+        <x:v>https://www.ralec.com/upload/media/product/file/IE-SP-010%20.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="62" customHeight="1">
@@ -3655,10 +3646,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D59" s="4" t="str">
-        <x:v>TPS22918DBVR</x:v>
+        <x:v>TPS22918DBVT</x:v>
       </x:c>
       <x:c r="E59" s="7" t="str">
-        <x:v>TPS22918DBVR</x:v>
+        <x:v>TPS22918DBVT</x:v>
       </x:c>
       <x:c r="F59" s="7" t="str">
         <x:v>Texas Instruments</x:v>
@@ -3670,7 +3661,7 @@
         <x:v>Active（原厂）</x:v>
       </x:c>
       <x:c r="I59" s="4" t="str">
-        <x:v>保持完整封装后缀与引脚定义</x:v>
+        <x:v>同TPS22918芯片及DBV6脚；T为250pcs小盘，ON/CT网络不变；2026-10-30嘉立创需订货（渠道快照，库存/交期下单复核）</x:v>
       </x:c>
       <x:c r="J59" s="4" t="str">
         <x:v>https://www.ti.com/product/TPS22918</x:v>
@@ -3946,7 +3937,7 @@
         <x:v>1uF</x:v>
       </x:c>
       <x:c r="E68" s="7" t="str">
-        <x:v>GRM188R71A105KA61D</x:v>
+        <x:v>GRM188R71E105KA12D</x:v>
       </x:c>
       <x:c r="F68" s="7" t="str">
         <x:v>Murata</x:v>
@@ -3958,10 +3949,10 @@
         <x:v>原理图已选完整MPN</x:v>
       </x:c>
       <x:c r="I68" s="4" t="str">
-        <x:v>MLCC标称值不代表工作偏压下有效值</x:v>
+        <x:v>25V/1uF/X7R±10%/0603；5V本地旁路，与MainBoard:C24同料C86020，各焊1颗；供电与热插拔须实测</x:v>
       </x:c>
       <x:c r="J68" s="4" t="str">
-        <x:v>https://ds.murata.com/simserve/characteristics?ReqType=TechPDF&amp;partnumber=GRM188R71A105KA61&amp;techpdfname=technical_pdf_Capacitor01&amp;lang=en</x:v>
+        <x:v>https://ds.murata.com/simserve/characteristics?ReqType=TechPDF&amp;partnumber=GRM188R71E105KA12&amp;techpdfname=technical_pdf_Capacitor01&amp;lang=en</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="62" customHeight="1">
@@ -4190,7 +4181,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b16560253fa498c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5c92056e36e4c33"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>